<commit_message>
removed TTBNP from original library from original annotatoons dude to likely mislable
</commit_message>
<xml_diff>
--- a/Outputs/Tables/T2.xlsx
+++ b/Outputs/Tables/T2.xlsx
@@ -23,7 +23,7 @@
     <t xml:space="preserve">AGROCHEMICALS</t>
   </si>
   <si>
-    <t xml:space="preserve">161 (36.3%)</t>
+    <t xml:space="preserve">161 (36.4%)</t>
   </si>
   <si>
     <t xml:space="preserve">    Insecticides and Pesticides</t>
@@ -206,7 +206,7 @@
     <t xml:space="preserve">POLLUTANTS AND INDUSTRIAL CHEMICALS</t>
   </si>
   <si>
-    <t xml:space="preserve">223 (50.3%)</t>
+    <t xml:space="preserve">222 (50.2%)</t>
   </si>
   <si>
     <t xml:space="preserve">    Chemical Synthesis Intermediates</t>
@@ -272,16 +272,16 @@
     <t xml:space="preserve">    Flame Retardants</t>
   </si>
   <si>
-    <t xml:space="preserve">17 (8%)</t>
+    <t xml:space="preserve">16 (7%)</t>
   </si>
   <si>
     <t xml:space="preserve">        Brominated</t>
   </si>
   <si>
-    <t xml:space="preserve">9 (53%)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4 (23.5%)</t>
+    <t xml:space="preserve">8 (50%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 (25%)</t>
   </si>
   <si>
     <t xml:space="preserve">        Organophosphate</t>

</xml_diff>

<commit_message>
Nomenclature, FDR analysis, Table 4 literature rebuild, and claim-validation script
</commit_message>
<xml_diff>
--- a/Outputs/Tables/T2.xlsx
+++ b/Outputs/Tables/T2.xlsx
@@ -14,7 +14,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="107">
   <si>
-    <t xml:space="preserve">GROUP: Class: Type</t>
+    <t xml:space="preserve">GROUP    Class        Type</t>
   </si>
   <si>
     <t xml:space="preserve">n (%)</t>
@@ -215,7 +215,7 @@
     <t xml:space="preserve">49 (22%)</t>
   </si>
   <si>
-    <t xml:space="preserve">    Dye intermediates</t>
+    <t xml:space="preserve">    Dye Intermediates</t>
   </si>
   <si>
     <t xml:space="preserve">37 (17%)</t>
@@ -337,7 +337,7 @@
 ¶ Includes the carbamate breakdown product, aldicarb sulfone
 ‖ Includes a triazinone (metribuzin)
 # Includes the wood preservative breakdown product, pentachloroanisole
-Abbreviations: UV = Ultraviolet</t>
+Abbreviations: UV = ultraviolet</t>
   </si>
 </sst>
 </file>
@@ -345,7 +345,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -369,6 +369,11 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
     </font>
   </fonts>
   <fills count="3">
@@ -424,7 +429,7 @@
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">

</xml_diff>